<commit_message>
Prepare tables to open
</commit_message>
<xml_diff>
--- a/outputs/gebaeudemodell/GebTyp/npro_type_mapping_GebTyp.xlsx
+++ b/outputs/gebaeudemodell/GebTyp/npro_type_mapping_GebTyp.xlsx
@@ -10,6 +10,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$C$15</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -31,52 +34,52 @@
     <t xml:space="preserve">npro_type</t>
   </si>
   <si>
+    <t xml:space="preserve">EFH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wohnen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">muss fachlich entschieden werden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MFH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B�ro-, Verwaltungs- oder Amtsgeb�ude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Büro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handelsgeb�ude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einzelhandel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produktions-, Werkstatt-, Lager- oder Betriebsgeb�ude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GMH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geb�ude f�r Kultur und Freizeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schule, Kindertagesst�tte und sonstiges Betreuungsgeb�ude</t>
+  </si>
+  <si>
     <t xml:space="preserve">Beherbergungs- oder Unterbringungsgeb�ude, Gastronomie- oder Verpflegungsgeb�ude</t>
   </si>
   <si>
-    <t xml:space="preserve">muss fachlich entschieden werden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B�ro-, Verwaltungs- oder Amtsgeb�ude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Büro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EFH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wohnen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GMH</t>
-  </si>
-  <si>
     <t xml:space="preserve">Geb�ude f�r Forschung und Hochschullehre</t>
   </si>
   <si>
     <t xml:space="preserve">Geb�ude f�r Gesundheit und Pflege</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geb�ude f�r Kultur und Freizeit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Handelsgeb�ude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einzelhandel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MFH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Produktions-, Werkstatt-, Lager- oder Betriebsgeb�ude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schule, Kindertagesst�tte und sonstiges Betreuungsgeb�ude</t>
   </si>
   <si>
     <t xml:space="preserve">Verkehrsgeb�ude</t>
@@ -169,12 +172,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -187,7 +194,28 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -373,174 +401,175 @@
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="78.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="78.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
+        <v>7946</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="1" t="n">
+        <v>2279</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>522</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>440</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>358</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>69</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="0" t="n">
-        <v>358</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="0" t="n">
-        <v>7946</v>
-      </c>
-      <c r="C4" s="0" t="s">
+      <c r="B10" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="1" t="n">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="0" t="n">
-        <v>52</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="0" t="n">
-        <v>39</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="0" t="n">
-        <v>69</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="n">
-        <v>2279</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="0" t="n">
-        <v>522</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="0" t="n">
-        <v>60</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="0" t="n">
-        <v>440</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="0" t="n">
-        <v>27</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>4</v>
+      <c r="C14" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>4</v>
+      <c r="B15" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C15"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -548,5 +577,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>